<commit_message>
cleanup: renombrar accionab→aplicab en hoja rubrica del Excel scored
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eval/rubrics/human_evaluation_comparative_scored.xlsx
+++ b/eval/rubrics/human_evaluation_comparative_scored.xlsx
@@ -5865,7 +5865,7 @@
     <row r="5" ht="150" customHeight="1" s="7">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>accionabilidad</t>
+          <t>aplicabilidad</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -5875,7 +5875,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>No ofrece pasos accionables.</t>
+          <t>No ofrece pasos aplicables.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -5895,7 +5895,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Procedimiento perfectamente accionable; sin ambigüedad, con canales y validaciones.</t>
+          <t>Procedimiento perfectamente aplicable; sin ambigüedad, con canales y validaciones.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -5942,10 +5942,11 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Ancla 5: cause='No aplica' en howto y resolution accionable; Ancla 1: problem habla de tarjetas y resolution de transferencias.</t>
-        </is>
-      </c>
-    </row>
+          <t>Ancla 5: cause='No aplica' en howto y resolution aplicable; Ancla 1: problem habla de tarjetas y resolution de transferencias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>

</xml_diff>